<commit_message>
Update Active Conduit Pool Tracking List 4.17.2026.xlsx
</commit_message>
<xml_diff>
--- a/Python/Active Conduit Pool Tracking List 4.17.2026.xlsx
+++ b/Python/Active Conduit Pool Tracking List 4.17.2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Lenders\Z. CMBS Test\6. CMBS Report - 10D Forms\Python\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gantryinc-my.sharepoint.com/personal/adowner_gantryinc_com/Documents/Documents/GitHub/10-D-Forms/Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{5BE99C24-D929-40C9-BD22-3D199804F4E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{1375740E-B79C-44E8-B58C-BFF393B47E38}"/>
+    <workbookView xWindow="32745" yWindow="3990" windowWidth="17280" windowHeight="9960" xr2:uid="{1375740E-B79C-44E8-B58C-BFF393B47E38}"/>
   </bookViews>
   <sheets>
     <sheet name="Active Pools" sheetId="1" r:id="rId1"/>

</xml_diff>